<commit_message>
feat: added hba1c, CAL and probing depth in the additional information
</commit_message>
<xml_diff>
--- a/backend/data_test/patients.xlsx
+++ b/backend/data_test/patients.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AK2"/>
+  <dimension ref="A1:AN1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
@@ -463,334 +463,162 @@
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
+          <t>HbA1c Level</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Clinical Attachment Level</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Probing Depth</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
           <t>Smoking</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Alcohol Consumption</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Chewing Habit</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Medical Condition</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Allergies</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>Date Created</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Last Updated</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>Right Thumb Image Path</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>Right Thumb Annotated Path</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>Right Index Image Path</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>Right Index Annotated Path</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>Right Middle Image Path</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>Right Middle Annotated Path</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>Right Ring Image Path</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>Right Ring Annotated Path</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>Right Little Image Path</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>Right Little Annotated Path</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>Left Thumb Image Path</t>
         </is>
       </c>
-      <c r="AC1" s="1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>Left Thumb Annotated Path</t>
         </is>
       </c>
-      <c r="AD1" s="1" t="inlineStr">
+      <c r="AG1" s="1" t="inlineStr">
         <is>
           <t>Left Index Image Path</t>
         </is>
       </c>
-      <c r="AE1" s="1" t="inlineStr">
+      <c r="AH1" s="1" t="inlineStr">
         <is>
           <t>Left Index Annotated Path</t>
         </is>
       </c>
-      <c r="AF1" s="1" t="inlineStr">
+      <c r="AI1" s="1" t="inlineStr">
         <is>
           <t>Left Middle Image Path</t>
         </is>
       </c>
-      <c r="AG1" s="1" t="inlineStr">
+      <c r="AJ1" s="1" t="inlineStr">
         <is>
           <t>Left Middle Annotated Path</t>
         </is>
       </c>
-      <c r="AH1" s="1" t="inlineStr">
+      <c r="AK1" s="1" t="inlineStr">
         <is>
           <t>Left Ring Image Path</t>
         </is>
       </c>
-      <c r="AI1" s="1" t="inlineStr">
+      <c r="AL1" s="1" t="inlineStr">
         <is>
           <t>Left Ring Annotated Path</t>
         </is>
       </c>
-      <c r="AJ1" s="1" t="inlineStr">
+      <c r="AM1" s="1" t="inlineStr">
         <is>
           <t>Left Little Image Path</t>
         </is>
       </c>
-      <c r="AK1" s="1" t="inlineStr">
+      <c r="AN1" s="1" t="inlineStr">
         <is>
           <t>Left Little Annotated Path</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>PAT0001</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>test-uuid-12345-abcde</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>John Doe Updated</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>30-40</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Male</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>9876543210</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>123 Bio Street</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>Occasional</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>Peanuts</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>Testing backend integration save.</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>2026-07-03T21:22:00.023143</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>2026-07-03T21:22:00.109854</t>
-        </is>
-      </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>IN_PROGRESS</t>
-        </is>
-      </c>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="S2" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="T2" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="U2" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="V2" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="W2" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="X2" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="Y2" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="Z2" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="AA2" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="AB2" t="inlineStr">
-        <is>
-          <t>C:\Users\athar\OneDrive\Desktop\M\LM-data-collection-app-main\backend\data_test\patients\test-uuid-12345-abcde\left_thumb.jpg</t>
-        </is>
-      </c>
-      <c r="AC2" t="inlineStr">
-        <is>
-          <t>C:\Users\athar\OneDrive\Desktop\M\LM-data-collection-app-main\backend\data_test\patients\test-uuid-12345-abcde\left_thumb_annotated.jpg</t>
-        </is>
-      </c>
-      <c r="AD2" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="AE2" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="AF2" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="AG2" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="AH2" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="AI2" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="AJ2" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="AK2" t="inlineStr">
-        <is>
-          <t>NA</t>
         </is>
       </c>
     </row>

</xml_diff>